<commit_message>
Final commit to GitHub - updating the excel file
</commit_message>
<xml_diff>
--- a/ExportedEstimate.xlsx
+++ b/ExportedEstimate.xlsx
@@ -62,7 +62,7 @@
     <t>Virtual Machine Scale Sets</t>
   </si>
   <si>
-    <t xml:space="preserve">3 A0 (1 Core, 0.75 GB RAM) x 730 Hours (Pay as you go), Linux,  (Pay as you go)</t>
+    <t xml:space="preserve">1 A0 (1 Core, 0.75 GB RAM) x 730 Hours (Pay as you go), Linux,  (Pay as you go)</t>
   </si>
   <si>
     <t>IP Addresses</t>
@@ -95,7 +95,7 @@
     <t>All prices shown are in Australia – Dollar ($) AUD. This is a summary estimate, not a quote. For up to date pricing information please visit https://azure.microsoft.com/pricing/calculator/</t>
   </si>
   <si>
-    <t>This estimate was created at 9/18/2026 3:42:21 AM UTC.</t>
+    <t>This estimate was created at 9/18/2026 4:07:36 AM UTC.</t>
   </si>
 </sst>
 </file>
@@ -407,7 +407,7 @@
         <v>16</v>
       </c>
       <c r="F5" s="5">
-        <v>73.08628241674198</v>
+        <v>24.362094138913996</v>
       </c>
       <c r="G5" s="5">
         <v>0</v>
@@ -615,7 +615,7 @@
       </c>
       <c r="E11" s="12"/>
       <c r="F11" s="15">
-        <v>105.41611624834874</v>
+        <v>56.691927970520759</v>
       </c>
       <c r="G11" s="15">
         <v>0</v>

</xml_diff>